<commit_message>
Atualiza├º├úo autom├ítica (05/03/2026 14:26:27,14)
</commit_message>
<xml_diff>
--- a/Canudos.xlsx
+++ b/Canudos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PLANILHAS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B012A78-34CF-4F09-BE70-C040368832F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2259A7AE-31C0-45C7-99B6-54B94C158276}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{2551C110-448D-4C8A-AC10-E46F4B669B16}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{2551C110-448D-4C8A-AC10-E46F4B669B16}"/>
   </bookViews>
   <sheets>
     <sheet name="ENCABEÇAMENTO" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="379" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="390" uniqueCount="90">
   <si>
     <t>OS</t>
   </si>
@@ -300,6 +300,12 @@
   </si>
   <si>
     <t>OBSERVAÇÃO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MAQUINA APRESENTA DEFEITO NO ROLO QUE PASSA AS ARTES PARA O CANUDO, ROLO RACHOU POR COMPLETO </t>
+  </si>
+  <si>
+    <t>05/03/20206</t>
   </si>
 </sst>
 </file>
@@ -641,6 +647,15 @@
     <xf numFmtId="0" fontId="7" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="14" fontId="5" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -650,33 +665,13 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="5" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="54">
+  <dxfs count="60">
     <dxf>
-      <border outline="0">
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-      </border>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -694,7 +689,18 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border outline="0">
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
     </dxf>
     <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -723,9 +729,6 @@
           <color indexed="64"/>
         </bottom>
       </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -769,6 +772,41 @@
       </border>
     </dxf>
     <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
       <font>
         <b/>
         <i/>
@@ -801,20 +839,6 @@
         </right>
         <top/>
         <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
       </border>
     </dxf>
     <dxf>
@@ -2866,13 +2890,13 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>4</xdr:col>
-      <xdr:colOff>133350</xdr:colOff>
+      <xdr:colOff>114300</xdr:colOff>
       <xdr:row>0</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
-      <xdr:colOff>1296262</xdr:colOff>
+      <xdr:colOff>1277212</xdr:colOff>
       <xdr:row>1</xdr:row>
       <xdr:rowOff>114300</xdr:rowOff>
     </xdr:to>
@@ -2903,7 +2927,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="6457950" y="0"/>
+          <a:off x="6438900" y="0"/>
           <a:ext cx="1162912" cy="790575"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -2917,84 +2941,84 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{5BB2D3F9-C887-4B4C-B99D-D2DF65DEC2A6}" name="Tabela5" displayName="Tabela5" ref="A1:H1048576" totalsRowCount="1" headerRowDxfId="53" dataDxfId="51" headerRowBorderDxfId="52">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{5BB2D3F9-C887-4B4C-B99D-D2DF65DEC2A6}" name="Tabela5" displayName="Tabela5" ref="A1:H1048576" totalsRowCount="1" headerRowDxfId="59" dataDxfId="57" headerRowBorderDxfId="58">
   <autoFilter ref="A1:H1048575" xr:uid="{5BB2D3F9-C887-4B4C-B99D-D2DF65DEC2A6}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{087A0113-3A7F-4ED4-85E5-B6DA7A785E6E}" name="Data" dataDxfId="50" totalsRowDxfId="49"/>
-    <tableColumn id="2" xr3:uid="{B5ACDCB9-111C-4EEF-A7F2-0DFD4B46F701}" name="Turno" dataDxfId="48" totalsRowDxfId="47"/>
-    <tableColumn id="3" xr3:uid="{8DF57E4B-CE5D-4D81-A024-AF995D46B0D6}" name="OS" dataDxfId="46" totalsRowDxfId="45"/>
-    <tableColumn id="4" xr3:uid="{ED2D14F5-1612-4387-8474-BB902D6983C6}" name="Operador" dataDxfId="44" totalsRowDxfId="43"/>
-    <tableColumn id="5" xr3:uid="{98386C95-9775-4F1F-A3CC-9A16E030AF66}" name="Produzidos" dataDxfId="42" totalsRowDxfId="41"/>
-    <tableColumn id="6" xr3:uid="{3F049097-8486-4DDD-93F7-CCC691CC4860}" name="Perdas" dataDxfId="40" totalsRowDxfId="39"/>
-    <tableColumn id="7" xr3:uid="{26B92E51-FF95-433C-9069-C56C7828476A}" name="Observação" dataDxfId="38" totalsRowDxfId="37"/>
-    <tableColumn id="8" xr3:uid="{8B43B335-323F-4C61-82F4-07648230810B}" name="Coluna1" dataDxfId="36" totalsRowDxfId="35"/>
+    <tableColumn id="1" xr3:uid="{087A0113-3A7F-4ED4-85E5-B6DA7A785E6E}" name="Data" dataDxfId="56" totalsRowDxfId="55"/>
+    <tableColumn id="2" xr3:uid="{B5ACDCB9-111C-4EEF-A7F2-0DFD4B46F701}" name="Turno" dataDxfId="54" totalsRowDxfId="53"/>
+    <tableColumn id="3" xr3:uid="{8DF57E4B-CE5D-4D81-A024-AF995D46B0D6}" name="OS" dataDxfId="52" totalsRowDxfId="51"/>
+    <tableColumn id="4" xr3:uid="{ED2D14F5-1612-4387-8474-BB902D6983C6}" name="Operador" dataDxfId="50" totalsRowDxfId="49"/>
+    <tableColumn id="5" xr3:uid="{98386C95-9775-4F1F-A3CC-9A16E030AF66}" name="Produzidos" dataDxfId="48" totalsRowDxfId="47"/>
+    <tableColumn id="6" xr3:uid="{3F049097-8486-4DDD-93F7-CCC691CC4860}" name="Perdas" dataDxfId="46" totalsRowDxfId="45"/>
+    <tableColumn id="7" xr3:uid="{26B92E51-FF95-433C-9069-C56C7828476A}" name="Observação" dataDxfId="44" totalsRowDxfId="43"/>
+    <tableColumn id="8" xr3:uid="{8B43B335-323F-4C61-82F4-07648230810B}" name="Coluna1" dataDxfId="42" totalsRowDxfId="41"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{89285ECA-F282-4F01-A009-CC89A51CDC7A}" name="Tabela1" displayName="Tabela1" ref="N1:Q27" headerRowDxfId="34" dataDxfId="32" headerRowBorderDxfId="33">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{89285ECA-F282-4F01-A009-CC89A51CDC7A}" name="Tabela1" displayName="Tabela1" ref="N1:Q27" headerRowDxfId="40" dataDxfId="38" headerRowBorderDxfId="39">
   <autoFilter ref="N1:Q27" xr:uid="{89285ECA-F282-4F01-A009-CC89A51CDC7A}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{EDE6611D-5889-4C5E-8516-947DDEFF7DCC}" name="CANUDOS " totalsRowLabel="Total" dataDxfId="31" totalsRowDxfId="30"/>
-    <tableColumn id="2" xr3:uid="{7D1A3E97-C617-4FD2-B05B-A97B6AD5F90C}" name="CORES" dataDxfId="29" totalsRowDxfId="28"/>
-    <tableColumn id="3" xr3:uid="{03E79F60-8E38-46EF-92B4-918A623037DE}" name="DESCRIÇÃO" totalsRowFunction="count" dataDxfId="27"/>
-    <tableColumn id="4" xr3:uid="{1B33BBDF-2D4E-45C0-873F-D04B114DCBBF}" name="os" dataDxfId="26"/>
+    <tableColumn id="1" xr3:uid="{EDE6611D-5889-4C5E-8516-947DDEFF7DCC}" name="CANUDOS " totalsRowLabel="Total" dataDxfId="37" totalsRowDxfId="36"/>
+    <tableColumn id="2" xr3:uid="{7D1A3E97-C617-4FD2-B05B-A97B6AD5F90C}" name="CORES" dataDxfId="35" totalsRowDxfId="34"/>
+    <tableColumn id="3" xr3:uid="{03E79F60-8E38-46EF-92B4-918A623037DE}" name="DESCRIÇÃO" totalsRowFunction="count" dataDxfId="33"/>
+    <tableColumn id="4" xr3:uid="{1B33BBDF-2D4E-45C0-873F-D04B114DCBBF}" name="os" dataDxfId="32"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{1FE77D6E-600C-406D-AA64-535CF7AD02D9}" name="Tabela4" displayName="Tabela4" ref="R2:S5" totalsRowShown="0" headerRowDxfId="25" dataDxfId="23" headerRowBorderDxfId="24">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{1FE77D6E-600C-406D-AA64-535CF7AD02D9}" name="Tabela4" displayName="Tabela4" ref="R2:S5" totalsRowShown="0" headerRowDxfId="31" dataDxfId="29" headerRowBorderDxfId="30">
   <autoFilter ref="R2:S5" xr:uid="{1FE77D6E-600C-406D-AA64-535CF7AD02D9}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{065934BB-F4F9-47CC-8C25-186E2F5FD276}" name="NOME" dataDxfId="22"/>
-    <tableColumn id="2" xr3:uid="{5F9476BD-3CB7-480B-BA25-725A0FDEB9A9}" name="RAMAL" dataDxfId="21"/>
+    <tableColumn id="1" xr3:uid="{065934BB-F4F9-47CC-8C25-186E2F5FD276}" name="NOME" dataDxfId="28"/>
+    <tableColumn id="2" xr3:uid="{5F9476BD-3CB7-480B-BA25-725A0FDEB9A9}" name="RAMAL" dataDxfId="27"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{CA95B68F-F434-4033-BFD9-2BB1AA7C7BF7}" name="Tabela3" displayName="Tabela3" ref="A1:G1048576" totalsRowShown="0" headerRowDxfId="18" headerRowBorderDxfId="19" tableBorderDxfId="20">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{CA95B68F-F434-4033-BFD9-2BB1AA7C7BF7}" name="Tabela3" displayName="Tabela3" ref="A1:G1048576" totalsRowShown="0" headerRowDxfId="26" headerRowBorderDxfId="25" tableBorderDxfId="24">
   <autoFilter ref="A1:G1048576" xr:uid="{CA95B68F-F434-4033-BFD9-2BB1AA7C7BF7}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{0280B923-DB87-4E28-A2B5-2ABF26E67A3C}" name="Data" dataDxfId="8"/>
-    <tableColumn id="2" xr3:uid="{CDEDA308-953F-46E8-8272-8EB68D248564}" name="Turno" dataDxfId="7"/>
-    <tableColumn id="3" xr3:uid="{A09724A8-B36D-4AD5-98B7-ADD526A91EFB}" name="OS" dataDxfId="6"/>
-    <tableColumn id="4" xr3:uid="{AF64C0A2-C8AC-47A7-BF73-70D43293AAAA}" name="Operador" dataDxfId="5"/>
-    <tableColumn id="5" xr3:uid="{F74EB60A-3874-4909-8B14-62AD3728B999}" name="Produzidos" dataDxfId="4"/>
-    <tableColumn id="6" xr3:uid="{124854EA-F6BE-4A3F-B8F0-8D4078EF15EC}" name="Perdas" dataDxfId="3"/>
-    <tableColumn id="7" xr3:uid="{FAD2623B-15B5-49D0-88AC-906319948EA0}" name="Observação" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{0280B923-DB87-4E28-A2B5-2ABF26E67A3C}" name="Data" dataDxfId="23"/>
+    <tableColumn id="2" xr3:uid="{CDEDA308-953F-46E8-8272-8EB68D248564}" name="Turno" dataDxfId="22"/>
+    <tableColumn id="3" xr3:uid="{A09724A8-B36D-4AD5-98B7-ADD526A91EFB}" name="OS" dataDxfId="21"/>
+    <tableColumn id="4" xr3:uid="{AF64C0A2-C8AC-47A7-BF73-70D43293AAAA}" name="Operador" dataDxfId="20"/>
+    <tableColumn id="5" xr3:uid="{F74EB60A-3874-4909-8B14-62AD3728B999}" name="Produzidos" dataDxfId="19"/>
+    <tableColumn id="6" xr3:uid="{124854EA-F6BE-4A3F-B8F0-8D4078EF15EC}" name="Perdas" dataDxfId="18"/>
+    <tableColumn id="7" xr3:uid="{FAD2623B-15B5-49D0-88AC-906319948EA0}" name="Observação" dataDxfId="17"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{7C61B123-99B4-407D-925F-D62D7C54D232}" name="Tabela17" displayName="Tabela17" ref="N1:Q27" headerRowDxfId="17" dataDxfId="16" headerRowBorderDxfId="15">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{7C61B123-99B4-407D-925F-D62D7C54D232}" name="Tabela17" displayName="Tabela17" ref="N1:Q27" headerRowDxfId="16" dataDxfId="14" headerRowBorderDxfId="15">
   <autoFilter ref="N1:Q27" xr:uid="{7C61B123-99B4-407D-925F-D62D7C54D232}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{E76169FA-FCD1-44CA-96FF-791C61B530A3}" name="CANUDOS " totalsRowLabel="Total" dataDxfId="13" totalsRowDxfId="14"/>
-    <tableColumn id="2" xr3:uid="{35FFF8DF-05B8-44FE-B351-F847EE90084A}" name="CORES" dataDxfId="11" totalsRowDxfId="12"/>
-    <tableColumn id="3" xr3:uid="{9A289D66-8372-477D-979D-D9E4A4CA121C}" name="DESCRIÇÃO" totalsRowFunction="count" dataDxfId="10"/>
-    <tableColumn id="4" xr3:uid="{0D9D8711-FBB3-4387-B4D2-D3D4718A6B6D}" name="os" dataDxfId="9"/>
+    <tableColumn id="1" xr3:uid="{E76169FA-FCD1-44CA-96FF-791C61B530A3}" name="CANUDOS " totalsRowLabel="Total" dataDxfId="13" totalsRowDxfId="12"/>
+    <tableColumn id="2" xr3:uid="{35FFF8DF-05B8-44FE-B351-F847EE90084A}" name="CORES" dataDxfId="11" totalsRowDxfId="10"/>
+    <tableColumn id="3" xr3:uid="{9A289D66-8372-477D-979D-D9E4A4CA121C}" name="DESCRIÇÃO" totalsRowFunction="count" dataDxfId="9"/>
+    <tableColumn id="4" xr3:uid="{0D9D8711-FBB3-4387-B4D2-D3D4718A6B6D}" name="os" dataDxfId="8"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{B6F26BC4-2F5B-4DD0-B255-2DBF5E945A60}" name="Tabela7" displayName="Tabela7" ref="A1:E1048576" totalsRowShown="0" headerRowBorderDxfId="0" tableBorderDxfId="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{B6F26BC4-2F5B-4DD0-B255-2DBF5E945A60}" name="Tabela7" displayName="Tabela7" ref="A1:E1048576" totalsRowShown="0" dataDxfId="1" headerRowBorderDxfId="7" tableBorderDxfId="6">
   <autoFilter ref="A1:E1048576" xr:uid="{B6F26BC4-2F5B-4DD0-B255-2DBF5E945A60}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{A457A19A-4874-4397-B513-B6F9A3B0A60A}" name="Data"/>
-    <tableColumn id="2" xr3:uid="{95C69B8D-1A39-40CB-B5FA-F58DC3500DA7}" name="Turno"/>
-    <tableColumn id="3" xr3:uid="{046BEC21-BC63-4C71-8608-9399078C3481}" name="OPERADOR"/>
-    <tableColumn id="4" xr3:uid="{C3B0A1FD-B664-4E6E-9624-C807349AADDB}" name="OBSERVAÇÃO"/>
-    <tableColumn id="5" xr3:uid="{C7967862-84A2-4EDD-9459-5C2DFCE69540}" name="Coluna1"/>
+    <tableColumn id="1" xr3:uid="{A457A19A-4874-4397-B513-B6F9A3B0A60A}" name="Data" dataDxfId="5"/>
+    <tableColumn id="2" xr3:uid="{95C69B8D-1A39-40CB-B5FA-F58DC3500DA7}" name="Turno" dataDxfId="4"/>
+    <tableColumn id="3" xr3:uid="{046BEC21-BC63-4C71-8608-9399078C3481}" name="OPERADOR" dataDxfId="3"/>
+    <tableColumn id="4" xr3:uid="{C3B0A1FD-B664-4E6E-9624-C807349AADDB}" name="OBSERVAÇÃO" dataDxfId="0"/>
+    <tableColumn id="5" xr3:uid="{C7967862-84A2-4EDD-9459-5C2DFCE69540}" name="Coluna1" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3344,11 +3368,11 @@
       <c r="J1" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="K1" s="29" t="s">
+      <c r="K1" s="32" t="s">
         <v>12</v>
       </c>
-      <c r="L1" s="29"/>
-      <c r="M1" s="29"/>
+      <c r="L1" s="32"/>
+      <c r="M1" s="32"/>
       <c r="N1" s="15" t="s">
         <v>24</v>
       </c>
@@ -3361,10 +3385,10 @@
       <c r="Q1" s="19" t="s">
         <v>55</v>
       </c>
-      <c r="R1" s="30" t="s">
+      <c r="R1" s="33" t="s">
         <v>56</v>
       </c>
-      <c r="S1" s="31"/>
+      <c r="S1" s="34"/>
     </row>
     <row r="2" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A2" s="2">
@@ -6288,25 +6312,25 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="54" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="32" t="s">
+      <c r="A1" s="29" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="33" t="s">
+      <c r="B1" s="30" t="s">
         <v>4</v>
       </c>
-      <c r="C1" s="33" t="s">
+      <c r="C1" s="30" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="33" t="s">
+      <c r="D1" s="30" t="s">
         <v>5</v>
       </c>
-      <c r="E1" s="33" t="s">
+      <c r="E1" s="30" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="33" t="s">
+      <c r="F1" s="30" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="33" t="s">
+      <c r="G1" s="30" t="s">
         <v>10</v>
       </c>
       <c r="H1" s="28" t="s">
@@ -6318,11 +6342,11 @@
       <c r="J1" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="K1" s="29" t="s">
+      <c r="K1" s="32" t="s">
         <v>12</v>
       </c>
-      <c r="L1" s="29"/>
-      <c r="M1" s="29"/>
+      <c r="L1" s="32"/>
+      <c r="M1" s="32"/>
       <c r="N1" s="15" t="s">
         <v>24</v>
       </c>
@@ -6364,7 +6388,7 @@
       <c r="I2" s="13"/>
       <c r="J2" s="14">
         <f>AVERAGE(E2:E206)</f>
-        <v>3200</v>
+        <v>2600</v>
       </c>
       <c r="K2" s="6" t="s">
         <v>13</v>
@@ -6385,16 +6409,40 @@
       <c r="Q2" s="1"/>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A3" s="2">
+        <v>46085</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3" s="1">
+        <v>1406169</v>
+      </c>
+      <c r="D3" s="1">
+        <v>8524</v>
+      </c>
+      <c r="E3" s="1">
+        <v>2000</v>
+      </c>
+      <c r="F3" s="1">
+        <v>200</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="H3" t="s">
+        <v>17</v>
+      </c>
       <c r="I3" s="12"/>
       <c r="J3" s="1"/>
       <c r="K3" s="4">
         <f>SUM(E2:E2000)</f>
-        <v>3200</v>
+        <v>5200</v>
       </c>
       <c r="L3" s="4"/>
       <c r="M3" s="18">
         <f>SUM(F2:F2000)</f>
-        <v>200</v>
+        <v>400</v>
       </c>
       <c r="N3" s="1" t="s">
         <v>27</v>
@@ -6410,6 +6458,24 @@
       </c>
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A4" s="2">
+        <v>46086</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D4" s="1">
+        <v>8524</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="H4" t="s">
+        <v>17</v>
+      </c>
       <c r="I4" s="4">
         <f>I2+I3</f>
         <v>0</v>
@@ -6728,28 +6794,45 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A6B5184B-1E33-47EF-9675-0892F220B5E2}">
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="4" width="23.7109375" customWidth="1"/>
-    <col min="5" max="5" width="21.5703125" customWidth="1"/>
+    <col min="1" max="4" width="23.7109375" style="1" customWidth="1"/>
+    <col min="5" max="5" width="21.5703125" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="53.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="32" t="s">
+      <c r="A1" s="29" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="33" t="s">
+      <c r="B1" s="30" t="s">
         <v>4</v>
       </c>
-      <c r="C1" s="33" t="s">
+      <c r="C1" s="30" t="s">
         <v>86</v>
       </c>
-      <c r="D1" s="32" t="s">
+      <c r="D1" s="29" t="s">
         <v>87</v>
       </c>
-      <c r="E1" s="34" t="s">
+      <c r="E1" s="31" t="s">
         <v>18</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" s="1">
+        <v>8524</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>17</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualiza├º├úo autom├ítica (09/03/2026 11:51:40,47)
</commit_message>
<xml_diff>
--- a/Canudos.xlsx
+++ b/Canudos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PLANILHAS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2259A7AE-31C0-45C7-99B6-54B94C158276}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{766FECA2-ED9B-495E-898D-877A07362EA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{2551C110-448D-4C8A-AC10-E46F4B669B16}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{2551C110-448D-4C8A-AC10-E46F4B669B16}"/>
   </bookViews>
   <sheets>
     <sheet name="ENCABEÇAMENTO" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="390" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="393" uniqueCount="91">
   <si>
     <t>OS</t>
   </si>
@@ -306,6 +306,9 @@
   </si>
   <si>
     <t>05/03/20206</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VOLTA DA MAQUINA 29, OPERADOR AUXILIOU NAS MAQUINAS DE IMPRESSÃO ENQUANTO OPERADOR DIEGO FAZIA TESTES E DPS TROCAVA MOLDE PARA NOVA ORDEM </t>
   </si>
 </sst>
 </file>
@@ -686,14 +689,14 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
       <border outline="0">
         <top style="thin">
           <color indexed="64"/>
         </top>
       </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <border outline="0">
@@ -3011,14 +3014,14 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{B6F26BC4-2F5B-4DD0-B255-2DBF5E945A60}" name="Tabela7" displayName="Tabela7" ref="A1:E1048576" totalsRowShown="0" dataDxfId="1" headerRowBorderDxfId="7" tableBorderDxfId="6">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{B6F26BC4-2F5B-4DD0-B255-2DBF5E945A60}" name="Tabela7" displayName="Tabela7" ref="A1:E1048576" totalsRowShown="0" dataDxfId="6" headerRowBorderDxfId="7" tableBorderDxfId="5">
   <autoFilter ref="A1:E1048576" xr:uid="{B6F26BC4-2F5B-4DD0-B255-2DBF5E945A60}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{A457A19A-4874-4397-B513-B6F9A3B0A60A}" name="Data" dataDxfId="5"/>
-    <tableColumn id="2" xr3:uid="{95C69B8D-1A39-40CB-B5FA-F58DC3500DA7}" name="Turno" dataDxfId="4"/>
-    <tableColumn id="3" xr3:uid="{046BEC21-BC63-4C71-8608-9399078C3481}" name="OPERADOR" dataDxfId="3"/>
-    <tableColumn id="4" xr3:uid="{C3B0A1FD-B664-4E6E-9624-C807349AADDB}" name="OBSERVAÇÃO" dataDxfId="0"/>
-    <tableColumn id="5" xr3:uid="{C7967862-84A2-4EDD-9459-5C2DFCE69540}" name="Coluna1" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{A457A19A-4874-4397-B513-B6F9A3B0A60A}" name="Data" dataDxfId="4"/>
+    <tableColumn id="2" xr3:uid="{95C69B8D-1A39-40CB-B5FA-F58DC3500DA7}" name="Turno" dataDxfId="3"/>
+    <tableColumn id="3" xr3:uid="{046BEC21-BC63-4C71-8608-9399078C3481}" name="OPERADOR" dataDxfId="2"/>
+    <tableColumn id="4" xr3:uid="{C3B0A1FD-B664-4E6E-9624-C807349AADDB}" name="OBSERVAÇÃO" dataDxfId="1"/>
+    <tableColumn id="5" xr3:uid="{C7967862-84A2-4EDD-9459-5C2DFCE69540}" name="Coluna1" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -6388,7 +6391,7 @@
       <c r="I2" s="13"/>
       <c r="J2" s="14">
         <f>AVERAGE(E2:E206)</f>
-        <v>2600</v>
+        <v>1854.6666666666667</v>
       </c>
       <c r="K2" s="6" t="s">
         <v>13</v>
@@ -6437,12 +6440,12 @@
       <c r="J3" s="1"/>
       <c r="K3" s="4">
         <f>SUM(E2:E2000)</f>
-        <v>5200</v>
+        <v>5564</v>
       </c>
       <c r="L3" s="4"/>
       <c r="M3" s="18">
         <f>SUM(F2:F2000)</f>
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="N3" s="1" t="s">
         <v>27</v>
@@ -6496,6 +6499,30 @@
       <c r="Q4" s="1"/>
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A5" s="2">
+        <v>46087</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C5" s="1">
+        <v>1406169</v>
+      </c>
+      <c r="D5" s="1">
+        <v>8524</v>
+      </c>
+      <c r="E5" s="1">
+        <v>364</v>
+      </c>
+      <c r="F5" s="1">
+        <v>100</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="H5" t="s">
+        <v>17</v>
+      </c>
       <c r="N5" s="1" t="s">
         <v>27</v>
       </c>

</xml_diff>

<commit_message>
Atualiza├º├úo autom├ítica (10/03/2026  8:27:42,55)
</commit_message>
<xml_diff>
--- a/Canudos.xlsx
+++ b/Canudos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PLANILHAS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{766FECA2-ED9B-495E-898D-877A07362EA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D55609FD-14FE-44B6-BBD8-F114A48F4762}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{2551C110-448D-4C8A-AC10-E46F4B669B16}"/>
+    <workbookView xWindow="2895" yWindow="2895" windowWidth="21600" windowHeight="11295" activeTab="1" xr2:uid="{2551C110-448D-4C8A-AC10-E46F4B669B16}"/>
   </bookViews>
   <sheets>
     <sheet name="ENCABEÇAMENTO" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="393" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="396" uniqueCount="92">
   <si>
     <t>OS</t>
   </si>
@@ -309,6 +309,9 @@
   </si>
   <si>
     <t xml:space="preserve">VOLTA DA MAQUINA 29, OPERADOR AUXILIOU NAS MAQUINAS DE IMPRESSÃO ENQUANTO OPERADOR DIEGO FAZIA TESTES E DPS TROCAVA MOLDE PARA NOVA ORDEM </t>
+  </si>
+  <si>
+    <t xml:space="preserve">MAQUINA NÃO APRESENTOU PROBLEMAS </t>
   </si>
 </sst>
 </file>
@@ -6391,7 +6394,7 @@
       <c r="I2" s="13"/>
       <c r="J2" s="14">
         <f>AVERAGE(E2:E206)</f>
-        <v>1854.6666666666667</v>
+        <v>1809</v>
       </c>
       <c r="K2" s="6" t="s">
         <v>13</v>
@@ -6440,12 +6443,12 @@
       <c r="J3" s="1"/>
       <c r="K3" s="4">
         <f>SUM(E2:E2000)</f>
-        <v>5564</v>
+        <v>7236</v>
       </c>
       <c r="L3" s="4"/>
       <c r="M3" s="18">
         <f>SUM(F2:F2000)</f>
-        <v>500</v>
+        <v>573</v>
       </c>
       <c r="N3" s="1" t="s">
         <v>27</v>
@@ -6535,6 +6538,30 @@
       <c r="Q5" s="1"/>
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A6" s="2">
+        <v>46090</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C6" s="1">
+        <v>1406169</v>
+      </c>
+      <c r="D6" s="1">
+        <v>8524</v>
+      </c>
+      <c r="E6" s="1">
+        <v>1672</v>
+      </c>
+      <c r="F6" s="1">
+        <v>73</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="H6" t="s">
+        <v>17</v>
+      </c>
       <c r="N6" s="1" t="s">
         <v>27</v>
       </c>

</xml_diff>

<commit_message>
Atualizacao automatica (13/03/2026 11:37:22,65)
</commit_message>
<xml_diff>
--- a/Canudos.xlsx
+++ b/Canudos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PLANILHAS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D55609FD-14FE-44B6-BBD8-F114A48F4762}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8014870D-DF73-44E0-B600-012863E04805}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2895" yWindow="2895" windowWidth="21600" windowHeight="11295" activeTab="1" xr2:uid="{2551C110-448D-4C8A-AC10-E46F4B669B16}"/>
+    <workbookView xWindow="2895" yWindow="2895" windowWidth="21600" windowHeight="11295" activeTab="2" xr2:uid="{2551C110-448D-4C8A-AC10-E46F4B669B16}"/>
   </bookViews>
   <sheets>
     <sheet name="ENCABEÇAMENTO" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="396" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="401" uniqueCount="93">
   <si>
     <t>OS</t>
   </si>
@@ -305,13 +305,16 @@
     <t xml:space="preserve">MAQUINA APRESENTA DEFEITO NO ROLO QUE PASSA AS ARTES PARA O CANUDO, ROLO RACHOU POR COMPLETO </t>
   </si>
   <si>
-    <t>05/03/20206</t>
-  </si>
-  <si>
     <t xml:space="preserve">VOLTA DA MAQUINA 29, OPERADOR AUXILIOU NAS MAQUINAS DE IMPRESSÃO ENQUANTO OPERADOR DIEGO FAZIA TESTES E DPS TROCAVA MOLDE PARA NOVA ORDEM </t>
   </si>
   <si>
     <t xml:space="preserve">MAQUINA NÃO APRESENTOU PROBLEMAS </t>
+  </si>
+  <si>
+    <t>MAQUINA APRESENTA DEFEITO NA ARTE (MINNIE ROSA), FORAM FEITOS VARIOS TESTES  AJUSTES, MAS O DEFEITO PERMANECEU, POSSIVEL PROBLEMA NO TRANSFER</t>
+  </si>
+  <si>
+    <t>MAQUINA APRESENTA DEFEITO NA ARTE (MINNIE ROSA), FORAM FEITOS VARIOS TESTES E AJUSTES, MAS O DEFEITO PERMANECEU, POSSIVEL PROBLEMA NO TRANSFER</t>
   </si>
 </sst>
 </file>
@@ -710,145 +713,6 @@
     </dxf>
     <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <border>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="0"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="4" tint="-0.249977111117893"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="18"/>
-        <color theme="0"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="4" tint="-0.249977111117893"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
         <left/>
         <right style="thin">
@@ -1046,6 +910,145 @@
         <b/>
         <i/>
         <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="18"/>
+        <color theme="0"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="4" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <border>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="0"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="4" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
         <outline val="0"/>
         <shadow val="0"/>
         <u val="none"/>
@@ -2947,70 +2950,70 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{5BB2D3F9-C887-4B4C-B99D-D2DF65DEC2A6}" name="Tabela5" displayName="Tabela5" ref="A1:H1048576" totalsRowCount="1" headerRowDxfId="59" dataDxfId="57" headerRowBorderDxfId="58">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{5BB2D3F9-C887-4B4C-B99D-D2DF65DEC2A6}" name="Tabela5" displayName="Tabela5" ref="A1:H1048576" totalsRowCount="1" headerRowDxfId="40" dataDxfId="38" headerRowBorderDxfId="39">
   <autoFilter ref="A1:H1048575" xr:uid="{5BB2D3F9-C887-4B4C-B99D-D2DF65DEC2A6}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{087A0113-3A7F-4ED4-85E5-B6DA7A785E6E}" name="Data" dataDxfId="56" totalsRowDxfId="55"/>
-    <tableColumn id="2" xr3:uid="{B5ACDCB9-111C-4EEF-A7F2-0DFD4B46F701}" name="Turno" dataDxfId="54" totalsRowDxfId="53"/>
-    <tableColumn id="3" xr3:uid="{8DF57E4B-CE5D-4D81-A024-AF995D46B0D6}" name="OS" dataDxfId="52" totalsRowDxfId="51"/>
-    <tableColumn id="4" xr3:uid="{ED2D14F5-1612-4387-8474-BB902D6983C6}" name="Operador" dataDxfId="50" totalsRowDxfId="49"/>
-    <tableColumn id="5" xr3:uid="{98386C95-9775-4F1F-A3CC-9A16E030AF66}" name="Produzidos" dataDxfId="48" totalsRowDxfId="47"/>
-    <tableColumn id="6" xr3:uid="{3F049097-8486-4DDD-93F7-CCC691CC4860}" name="Perdas" dataDxfId="46" totalsRowDxfId="45"/>
-    <tableColumn id="7" xr3:uid="{26B92E51-FF95-433C-9069-C56C7828476A}" name="Observação" dataDxfId="44" totalsRowDxfId="43"/>
-    <tableColumn id="8" xr3:uid="{8B43B335-323F-4C61-82F4-07648230810B}" name="Coluna1" dataDxfId="42" totalsRowDxfId="41"/>
+    <tableColumn id="1" xr3:uid="{087A0113-3A7F-4ED4-85E5-B6DA7A785E6E}" name="Data" dataDxfId="37" totalsRowDxfId="36"/>
+    <tableColumn id="2" xr3:uid="{B5ACDCB9-111C-4EEF-A7F2-0DFD4B46F701}" name="Turno" dataDxfId="35" totalsRowDxfId="34"/>
+    <tableColumn id="3" xr3:uid="{8DF57E4B-CE5D-4D81-A024-AF995D46B0D6}" name="OS" dataDxfId="33" totalsRowDxfId="32"/>
+    <tableColumn id="4" xr3:uid="{ED2D14F5-1612-4387-8474-BB902D6983C6}" name="Operador" dataDxfId="31" totalsRowDxfId="30"/>
+    <tableColumn id="5" xr3:uid="{98386C95-9775-4F1F-A3CC-9A16E030AF66}" name="Produzidos" dataDxfId="29" totalsRowDxfId="28"/>
+    <tableColumn id="6" xr3:uid="{3F049097-8486-4DDD-93F7-CCC691CC4860}" name="Perdas" dataDxfId="27" totalsRowDxfId="26"/>
+    <tableColumn id="7" xr3:uid="{26B92E51-FF95-433C-9069-C56C7828476A}" name="Observação" dataDxfId="25" totalsRowDxfId="24"/>
+    <tableColumn id="8" xr3:uid="{8B43B335-323F-4C61-82F4-07648230810B}" name="Coluna1" dataDxfId="23" totalsRowDxfId="22"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{89285ECA-F282-4F01-A009-CC89A51CDC7A}" name="Tabela1" displayName="Tabela1" ref="N1:Q27" headerRowDxfId="40" dataDxfId="38" headerRowBorderDxfId="39">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{89285ECA-F282-4F01-A009-CC89A51CDC7A}" name="Tabela1" displayName="Tabela1" ref="N1:Q27" headerRowDxfId="21" dataDxfId="19" headerRowBorderDxfId="20">
   <autoFilter ref="N1:Q27" xr:uid="{89285ECA-F282-4F01-A009-CC89A51CDC7A}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{EDE6611D-5889-4C5E-8516-947DDEFF7DCC}" name="CANUDOS " totalsRowLabel="Total" dataDxfId="37" totalsRowDxfId="36"/>
-    <tableColumn id="2" xr3:uid="{7D1A3E97-C617-4FD2-B05B-A97B6AD5F90C}" name="CORES" dataDxfId="35" totalsRowDxfId="34"/>
-    <tableColumn id="3" xr3:uid="{03E79F60-8E38-46EF-92B4-918A623037DE}" name="DESCRIÇÃO" totalsRowFunction="count" dataDxfId="33"/>
-    <tableColumn id="4" xr3:uid="{1B33BBDF-2D4E-45C0-873F-D04B114DCBBF}" name="os" dataDxfId="32"/>
+    <tableColumn id="1" xr3:uid="{EDE6611D-5889-4C5E-8516-947DDEFF7DCC}" name="CANUDOS " totalsRowLabel="Total" dataDxfId="18" totalsRowDxfId="17"/>
+    <tableColumn id="2" xr3:uid="{7D1A3E97-C617-4FD2-B05B-A97B6AD5F90C}" name="CORES" dataDxfId="16" totalsRowDxfId="15"/>
+    <tableColumn id="3" xr3:uid="{03E79F60-8E38-46EF-92B4-918A623037DE}" name="DESCRIÇÃO" totalsRowFunction="count" dataDxfId="14"/>
+    <tableColumn id="4" xr3:uid="{1B33BBDF-2D4E-45C0-873F-D04B114DCBBF}" name="os" dataDxfId="13"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{1FE77D6E-600C-406D-AA64-535CF7AD02D9}" name="Tabela4" displayName="Tabela4" ref="R2:S5" totalsRowShown="0" headerRowDxfId="31" dataDxfId="29" headerRowBorderDxfId="30">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{1FE77D6E-600C-406D-AA64-535CF7AD02D9}" name="Tabela4" displayName="Tabela4" ref="R2:S5" totalsRowShown="0" headerRowDxfId="12" dataDxfId="10" headerRowBorderDxfId="11">
   <autoFilter ref="R2:S5" xr:uid="{1FE77D6E-600C-406D-AA64-535CF7AD02D9}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{065934BB-F4F9-47CC-8C25-186E2F5FD276}" name="NOME" dataDxfId="28"/>
-    <tableColumn id="2" xr3:uid="{5F9476BD-3CB7-480B-BA25-725A0FDEB9A9}" name="RAMAL" dataDxfId="27"/>
+    <tableColumn id="1" xr3:uid="{065934BB-F4F9-47CC-8C25-186E2F5FD276}" name="NOME" dataDxfId="9"/>
+    <tableColumn id="2" xr3:uid="{5F9476BD-3CB7-480B-BA25-725A0FDEB9A9}" name="RAMAL" dataDxfId="8"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{CA95B68F-F434-4033-BFD9-2BB1AA7C7BF7}" name="Tabela3" displayName="Tabela3" ref="A1:G1048576" totalsRowShown="0" headerRowDxfId="26" headerRowBorderDxfId="25" tableBorderDxfId="24">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{CA95B68F-F434-4033-BFD9-2BB1AA7C7BF7}" name="Tabela3" displayName="Tabela3" ref="A1:G1048576" totalsRowShown="0" headerRowDxfId="59" headerRowBorderDxfId="58" tableBorderDxfId="57">
   <autoFilter ref="A1:G1048576" xr:uid="{CA95B68F-F434-4033-BFD9-2BB1AA7C7BF7}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{0280B923-DB87-4E28-A2B5-2ABF26E67A3C}" name="Data" dataDxfId="23"/>
-    <tableColumn id="2" xr3:uid="{CDEDA308-953F-46E8-8272-8EB68D248564}" name="Turno" dataDxfId="22"/>
-    <tableColumn id="3" xr3:uid="{A09724A8-B36D-4AD5-98B7-ADD526A91EFB}" name="OS" dataDxfId="21"/>
-    <tableColumn id="4" xr3:uid="{AF64C0A2-C8AC-47A7-BF73-70D43293AAAA}" name="Operador" dataDxfId="20"/>
-    <tableColumn id="5" xr3:uid="{F74EB60A-3874-4909-8B14-62AD3728B999}" name="Produzidos" dataDxfId="19"/>
-    <tableColumn id="6" xr3:uid="{124854EA-F6BE-4A3F-B8F0-8D4078EF15EC}" name="Perdas" dataDxfId="18"/>
-    <tableColumn id="7" xr3:uid="{FAD2623B-15B5-49D0-88AC-906319948EA0}" name="Observação" dataDxfId="17"/>
+    <tableColumn id="1" xr3:uid="{0280B923-DB87-4E28-A2B5-2ABF26E67A3C}" name="Data" dataDxfId="56"/>
+    <tableColumn id="2" xr3:uid="{CDEDA308-953F-46E8-8272-8EB68D248564}" name="Turno" dataDxfId="55"/>
+    <tableColumn id="3" xr3:uid="{A09724A8-B36D-4AD5-98B7-ADD526A91EFB}" name="OS" dataDxfId="54"/>
+    <tableColumn id="4" xr3:uid="{AF64C0A2-C8AC-47A7-BF73-70D43293AAAA}" name="Operador" dataDxfId="53"/>
+    <tableColumn id="5" xr3:uid="{F74EB60A-3874-4909-8B14-62AD3728B999}" name="Produzidos" dataDxfId="52"/>
+    <tableColumn id="6" xr3:uid="{124854EA-F6BE-4A3F-B8F0-8D4078EF15EC}" name="Perdas" dataDxfId="51"/>
+    <tableColumn id="7" xr3:uid="{FAD2623B-15B5-49D0-88AC-906319948EA0}" name="Observação" dataDxfId="50"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{7C61B123-99B4-407D-925F-D62D7C54D232}" name="Tabela17" displayName="Tabela17" ref="N1:Q27" headerRowDxfId="16" dataDxfId="14" headerRowBorderDxfId="15">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{7C61B123-99B4-407D-925F-D62D7C54D232}" name="Tabela17" displayName="Tabela17" ref="N1:Q27" headerRowDxfId="49" dataDxfId="47" headerRowBorderDxfId="48">
   <autoFilter ref="N1:Q27" xr:uid="{7C61B123-99B4-407D-925F-D62D7C54D232}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{E76169FA-FCD1-44CA-96FF-791C61B530A3}" name="CANUDOS " totalsRowLabel="Total" dataDxfId="13" totalsRowDxfId="12"/>
-    <tableColumn id="2" xr3:uid="{35FFF8DF-05B8-44FE-B351-F847EE90084A}" name="CORES" dataDxfId="11" totalsRowDxfId="10"/>
-    <tableColumn id="3" xr3:uid="{9A289D66-8372-477D-979D-D9E4A4CA121C}" name="DESCRIÇÃO" totalsRowFunction="count" dataDxfId="9"/>
-    <tableColumn id="4" xr3:uid="{0D9D8711-FBB3-4387-B4D2-D3D4718A6B6D}" name="os" dataDxfId="8"/>
+    <tableColumn id="1" xr3:uid="{E76169FA-FCD1-44CA-96FF-791C61B530A3}" name="CANUDOS " totalsRowLabel="Total" dataDxfId="46" totalsRowDxfId="45"/>
+    <tableColumn id="2" xr3:uid="{35FFF8DF-05B8-44FE-B351-F847EE90084A}" name="CORES" dataDxfId="44" totalsRowDxfId="43"/>
+    <tableColumn id="3" xr3:uid="{9A289D66-8372-477D-979D-D9E4A4CA121C}" name="DESCRIÇÃO" totalsRowFunction="count" dataDxfId="42"/>
+    <tableColumn id="4" xr3:uid="{0D9D8711-FBB3-4387-B4D2-D3D4718A6B6D}" name="os" dataDxfId="41"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -6394,7 +6397,7 @@
       <c r="I2" s="13"/>
       <c r="J2" s="14">
         <f>AVERAGE(E2:E206)</f>
-        <v>1809</v>
+        <v>1519.2</v>
       </c>
       <c r="K2" s="6" t="s">
         <v>13</v>
@@ -6443,12 +6446,12 @@
       <c r="J3" s="1"/>
       <c r="K3" s="4">
         <f>SUM(E2:E2000)</f>
-        <v>7236</v>
+        <v>7596</v>
       </c>
       <c r="L3" s="4"/>
       <c r="M3" s="18">
         <f>SUM(F2:F2000)</f>
-        <v>573</v>
+        <v>873</v>
       </c>
       <c r="N3" s="1" t="s">
         <v>27</v>
@@ -6521,7 +6524,7 @@
         <v>100</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="H5" t="s">
         <v>17</v>
@@ -6557,7 +6560,7 @@
         <v>73</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="H6" t="s">
         <v>17</v>
@@ -6576,6 +6579,30 @@
       </c>
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A7" s="2">
+        <v>46093</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C7" s="1">
+        <v>1406169</v>
+      </c>
+      <c r="D7" s="1">
+        <v>8524</v>
+      </c>
+      <c r="E7" s="1">
+        <v>360</v>
+      </c>
+      <c r="F7" s="1">
+        <v>300</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="H7" t="s">
+        <v>17</v>
+      </c>
       <c r="N7" s="1" t="s">
         <v>27</v>
       </c>
@@ -6848,7 +6875,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A6B5184B-1E33-47EF-9675-0892F220B5E2}">
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="4" width="23.7109375" style="1" customWidth="1"/>
@@ -6873,8 +6900,8 @@
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
-        <v>89</v>
+      <c r="A2" s="2">
+        <v>46086</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>6</v>
@@ -6886,6 +6913,23 @@
         <v>88</v>
       </c>
       <c r="E2" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" s="2">
+        <v>46093</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3" s="1">
+        <v>8524</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="E3" s="1" t="s">
         <v>17</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualizacao automatica (13/03/2026 16:02:46,93)
</commit_message>
<xml_diff>
--- a/Canudos.xlsx
+++ b/Canudos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PLANILHAS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8014870D-DF73-44E0-B600-012863E04805}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{943063A0-ED43-4A30-AA3E-9F44FCBA6D38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2895" yWindow="2895" windowWidth="21600" windowHeight="11295" activeTab="2" xr2:uid="{2551C110-448D-4C8A-AC10-E46F4B669B16}"/>
+    <workbookView xWindow="3585" yWindow="3585" windowWidth="21600" windowHeight="11295" xr2:uid="{2551C110-448D-4C8A-AC10-E46F4B669B16}"/>
   </bookViews>
   <sheets>
     <sheet name="ENCABEÇAMENTO" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="401" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="405" uniqueCount="94">
   <si>
     <t>OS</t>
   </si>
@@ -315,6 +315,9 @@
   </si>
   <si>
     <t>MAQUINA APRESENTA DEFEITO NA ARTE (MINNIE ROSA), FORAM FEITOS VARIOS TESTES E AJUSTES, MAS O DEFEITO PERMANECEU, POSSIVEL PROBLEMA NO TRANSFER</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RODANDO TRANSFER E ENCABEÇADORA </t>
   </si>
 </sst>
 </file>
@@ -695,6 +698,106 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <border>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="0"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="4" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <border outline="0">
         <top style="thin">
           <color indexed="64"/>
@@ -702,13 +805,45 @@
       </border>
     </dxf>
     <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
       <border outline="0">
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="18"/>
+        <color theme="0"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="4" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
       </border>
     </dxf>
     <dxf>
@@ -867,31 +1002,6 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
       <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -954,81 +1064,6 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <border>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="0"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="4" tint="-0.249977111117893"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
       <border outline="0">
         <top style="thin">
           <color indexed="64"/>
@@ -1036,45 +1071,13 @@
       </border>
     </dxf>
     <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <border outline="0">
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="18"/>
-        <color theme="0"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="4" tint="-0.249977111117893"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
       </border>
     </dxf>
   </dxfs>
@@ -2950,84 +2953,84 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{5BB2D3F9-C887-4B4C-B99D-D2DF65DEC2A6}" name="Tabela5" displayName="Tabela5" ref="A1:H1048576" totalsRowCount="1" headerRowDxfId="40" dataDxfId="38" headerRowBorderDxfId="39">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{5BB2D3F9-C887-4B4C-B99D-D2DF65DEC2A6}" name="Tabela5" displayName="Tabela5" ref="A1:H1048576" totalsRowCount="1" headerRowDxfId="51" dataDxfId="49" headerRowBorderDxfId="50">
   <autoFilter ref="A1:H1048575" xr:uid="{5BB2D3F9-C887-4B4C-B99D-D2DF65DEC2A6}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{087A0113-3A7F-4ED4-85E5-B6DA7A785E6E}" name="Data" dataDxfId="37" totalsRowDxfId="36"/>
-    <tableColumn id="2" xr3:uid="{B5ACDCB9-111C-4EEF-A7F2-0DFD4B46F701}" name="Turno" dataDxfId="35" totalsRowDxfId="34"/>
-    <tableColumn id="3" xr3:uid="{8DF57E4B-CE5D-4D81-A024-AF995D46B0D6}" name="OS" dataDxfId="33" totalsRowDxfId="32"/>
-    <tableColumn id="4" xr3:uid="{ED2D14F5-1612-4387-8474-BB902D6983C6}" name="Operador" dataDxfId="31" totalsRowDxfId="30"/>
-    <tableColumn id="5" xr3:uid="{98386C95-9775-4F1F-A3CC-9A16E030AF66}" name="Produzidos" dataDxfId="29" totalsRowDxfId="28"/>
-    <tableColumn id="6" xr3:uid="{3F049097-8486-4DDD-93F7-CCC691CC4860}" name="Perdas" dataDxfId="27" totalsRowDxfId="26"/>
-    <tableColumn id="7" xr3:uid="{26B92E51-FF95-433C-9069-C56C7828476A}" name="Observação" dataDxfId="25" totalsRowDxfId="24"/>
-    <tableColumn id="8" xr3:uid="{8B43B335-323F-4C61-82F4-07648230810B}" name="Coluna1" dataDxfId="23" totalsRowDxfId="22"/>
+    <tableColumn id="1" xr3:uid="{087A0113-3A7F-4ED4-85E5-B6DA7A785E6E}" name="Data" dataDxfId="48" totalsRowDxfId="7"/>
+    <tableColumn id="2" xr3:uid="{B5ACDCB9-111C-4EEF-A7F2-0DFD4B46F701}" name="Turno" dataDxfId="47" totalsRowDxfId="6"/>
+    <tableColumn id="3" xr3:uid="{8DF57E4B-CE5D-4D81-A024-AF995D46B0D6}" name="OS" dataDxfId="46" totalsRowDxfId="5"/>
+    <tableColumn id="4" xr3:uid="{ED2D14F5-1612-4387-8474-BB902D6983C6}" name="Operador" dataDxfId="45" totalsRowDxfId="4"/>
+    <tableColumn id="5" xr3:uid="{98386C95-9775-4F1F-A3CC-9A16E030AF66}" name="Produzidos" dataDxfId="44" totalsRowDxfId="3"/>
+    <tableColumn id="6" xr3:uid="{3F049097-8486-4DDD-93F7-CCC691CC4860}" name="Perdas" dataDxfId="43" totalsRowDxfId="2"/>
+    <tableColumn id="7" xr3:uid="{26B92E51-FF95-433C-9069-C56C7828476A}" name="Observação" dataDxfId="42" totalsRowDxfId="1"/>
+    <tableColumn id="8" xr3:uid="{8B43B335-323F-4C61-82F4-07648230810B}" name="Coluna1" dataDxfId="41" totalsRowDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{89285ECA-F282-4F01-A009-CC89A51CDC7A}" name="Tabela1" displayName="Tabela1" ref="N1:Q27" headerRowDxfId="21" dataDxfId="19" headerRowBorderDxfId="20">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{89285ECA-F282-4F01-A009-CC89A51CDC7A}" name="Tabela1" displayName="Tabela1" ref="N1:Q27" headerRowDxfId="40" dataDxfId="38" headerRowBorderDxfId="39">
   <autoFilter ref="N1:Q27" xr:uid="{89285ECA-F282-4F01-A009-CC89A51CDC7A}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{EDE6611D-5889-4C5E-8516-947DDEFF7DCC}" name="CANUDOS " totalsRowLabel="Total" dataDxfId="18" totalsRowDxfId="17"/>
-    <tableColumn id="2" xr3:uid="{7D1A3E97-C617-4FD2-B05B-A97B6AD5F90C}" name="CORES" dataDxfId="16" totalsRowDxfId="15"/>
-    <tableColumn id="3" xr3:uid="{03E79F60-8E38-46EF-92B4-918A623037DE}" name="DESCRIÇÃO" totalsRowFunction="count" dataDxfId="14"/>
-    <tableColumn id="4" xr3:uid="{1B33BBDF-2D4E-45C0-873F-D04B114DCBBF}" name="os" dataDxfId="13"/>
+    <tableColumn id="1" xr3:uid="{EDE6611D-5889-4C5E-8516-947DDEFF7DCC}" name="CANUDOS " totalsRowLabel="Total" dataDxfId="37" totalsRowDxfId="36"/>
+    <tableColumn id="2" xr3:uid="{7D1A3E97-C617-4FD2-B05B-A97B6AD5F90C}" name="CORES" dataDxfId="35" totalsRowDxfId="34"/>
+    <tableColumn id="3" xr3:uid="{03E79F60-8E38-46EF-92B4-918A623037DE}" name="DESCRIÇÃO" totalsRowFunction="count" dataDxfId="33"/>
+    <tableColumn id="4" xr3:uid="{1B33BBDF-2D4E-45C0-873F-D04B114DCBBF}" name="os" dataDxfId="32"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{1FE77D6E-600C-406D-AA64-535CF7AD02D9}" name="Tabela4" displayName="Tabela4" ref="R2:S5" totalsRowShown="0" headerRowDxfId="12" dataDxfId="10" headerRowBorderDxfId="11">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{1FE77D6E-600C-406D-AA64-535CF7AD02D9}" name="Tabela4" displayName="Tabela4" ref="R2:S5" totalsRowShown="0" headerRowDxfId="31" dataDxfId="29" headerRowBorderDxfId="30">
   <autoFilter ref="R2:S5" xr:uid="{1FE77D6E-600C-406D-AA64-535CF7AD02D9}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{065934BB-F4F9-47CC-8C25-186E2F5FD276}" name="NOME" dataDxfId="9"/>
-    <tableColumn id="2" xr3:uid="{5F9476BD-3CB7-480B-BA25-725A0FDEB9A9}" name="RAMAL" dataDxfId="8"/>
+    <tableColumn id="1" xr3:uid="{065934BB-F4F9-47CC-8C25-186E2F5FD276}" name="NOME" dataDxfId="28"/>
+    <tableColumn id="2" xr3:uid="{5F9476BD-3CB7-480B-BA25-725A0FDEB9A9}" name="RAMAL" dataDxfId="27"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{CA95B68F-F434-4033-BFD9-2BB1AA7C7BF7}" name="Tabela3" displayName="Tabela3" ref="A1:G1048576" totalsRowShown="0" headerRowDxfId="59" headerRowBorderDxfId="58" tableBorderDxfId="57">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{CA95B68F-F434-4033-BFD9-2BB1AA7C7BF7}" name="Tabela3" displayName="Tabela3" ref="A1:G1048576" totalsRowShown="0" headerRowDxfId="26" headerRowBorderDxfId="25" tableBorderDxfId="24">
   <autoFilter ref="A1:G1048576" xr:uid="{CA95B68F-F434-4033-BFD9-2BB1AA7C7BF7}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{0280B923-DB87-4E28-A2B5-2ABF26E67A3C}" name="Data" dataDxfId="56"/>
-    <tableColumn id="2" xr3:uid="{CDEDA308-953F-46E8-8272-8EB68D248564}" name="Turno" dataDxfId="55"/>
-    <tableColumn id="3" xr3:uid="{A09724A8-B36D-4AD5-98B7-ADD526A91EFB}" name="OS" dataDxfId="54"/>
-    <tableColumn id="4" xr3:uid="{AF64C0A2-C8AC-47A7-BF73-70D43293AAAA}" name="Operador" dataDxfId="53"/>
-    <tableColumn id="5" xr3:uid="{F74EB60A-3874-4909-8B14-62AD3728B999}" name="Produzidos" dataDxfId="52"/>
-    <tableColumn id="6" xr3:uid="{124854EA-F6BE-4A3F-B8F0-8D4078EF15EC}" name="Perdas" dataDxfId="51"/>
-    <tableColumn id="7" xr3:uid="{FAD2623B-15B5-49D0-88AC-906319948EA0}" name="Observação" dataDxfId="50"/>
+    <tableColumn id="1" xr3:uid="{0280B923-DB87-4E28-A2B5-2ABF26E67A3C}" name="Data" dataDxfId="23"/>
+    <tableColumn id="2" xr3:uid="{CDEDA308-953F-46E8-8272-8EB68D248564}" name="Turno" dataDxfId="22"/>
+    <tableColumn id="3" xr3:uid="{A09724A8-B36D-4AD5-98B7-ADD526A91EFB}" name="OS" dataDxfId="21"/>
+    <tableColumn id="4" xr3:uid="{AF64C0A2-C8AC-47A7-BF73-70D43293AAAA}" name="Operador" dataDxfId="20"/>
+    <tableColumn id="5" xr3:uid="{F74EB60A-3874-4909-8B14-62AD3728B999}" name="Produzidos" dataDxfId="19"/>
+    <tableColumn id="6" xr3:uid="{124854EA-F6BE-4A3F-B8F0-8D4078EF15EC}" name="Perdas" dataDxfId="18"/>
+    <tableColumn id="7" xr3:uid="{FAD2623B-15B5-49D0-88AC-906319948EA0}" name="Observação" dataDxfId="17"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{7C61B123-99B4-407D-925F-D62D7C54D232}" name="Tabela17" displayName="Tabela17" ref="N1:Q27" headerRowDxfId="49" dataDxfId="47" headerRowBorderDxfId="48">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{7C61B123-99B4-407D-925F-D62D7C54D232}" name="Tabela17" displayName="Tabela17" ref="N1:Q27" headerRowDxfId="16" dataDxfId="14" headerRowBorderDxfId="15">
   <autoFilter ref="N1:Q27" xr:uid="{7C61B123-99B4-407D-925F-D62D7C54D232}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{E76169FA-FCD1-44CA-96FF-791C61B530A3}" name="CANUDOS " totalsRowLabel="Total" dataDxfId="46" totalsRowDxfId="45"/>
-    <tableColumn id="2" xr3:uid="{35FFF8DF-05B8-44FE-B351-F847EE90084A}" name="CORES" dataDxfId="44" totalsRowDxfId="43"/>
-    <tableColumn id="3" xr3:uid="{9A289D66-8372-477D-979D-D9E4A4CA121C}" name="DESCRIÇÃO" totalsRowFunction="count" dataDxfId="42"/>
-    <tableColumn id="4" xr3:uid="{0D9D8711-FBB3-4387-B4D2-D3D4718A6B6D}" name="os" dataDxfId="41"/>
+    <tableColumn id="1" xr3:uid="{E76169FA-FCD1-44CA-96FF-791C61B530A3}" name="CANUDOS " totalsRowLabel="Total" dataDxfId="13" totalsRowDxfId="12"/>
+    <tableColumn id="2" xr3:uid="{35FFF8DF-05B8-44FE-B351-F847EE90084A}" name="CORES" dataDxfId="11" totalsRowDxfId="10"/>
+    <tableColumn id="3" xr3:uid="{9A289D66-8372-477D-979D-D9E4A4CA121C}" name="DESCRIÇÃO" totalsRowFunction="count" dataDxfId="9"/>
+    <tableColumn id="4" xr3:uid="{0D9D8711-FBB3-4387-B4D2-D3D4718A6B6D}" name="os" dataDxfId="8"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{B6F26BC4-2F5B-4DD0-B255-2DBF5E945A60}" name="Tabela7" displayName="Tabela7" ref="A1:E1048576" totalsRowShown="0" dataDxfId="6" headerRowBorderDxfId="7" tableBorderDxfId="5">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{B6F26BC4-2F5B-4DD0-B255-2DBF5E945A60}" name="Tabela7" displayName="Tabela7" ref="A1:E1048576" totalsRowShown="0" dataDxfId="58" headerRowBorderDxfId="59" tableBorderDxfId="57">
   <autoFilter ref="A1:E1048576" xr:uid="{B6F26BC4-2F5B-4DD0-B255-2DBF5E945A60}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{A457A19A-4874-4397-B513-B6F9A3B0A60A}" name="Data" dataDxfId="4"/>
-    <tableColumn id="2" xr3:uid="{95C69B8D-1A39-40CB-B5FA-F58DC3500DA7}" name="Turno" dataDxfId="3"/>
-    <tableColumn id="3" xr3:uid="{046BEC21-BC63-4C71-8608-9399078C3481}" name="OPERADOR" dataDxfId="2"/>
-    <tableColumn id="4" xr3:uid="{C3B0A1FD-B664-4E6E-9624-C807349AADDB}" name="OBSERVAÇÃO" dataDxfId="1"/>
-    <tableColumn id="5" xr3:uid="{C7967862-84A2-4EDD-9459-5C2DFCE69540}" name="Coluna1" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{A457A19A-4874-4397-B513-B6F9A3B0A60A}" name="Data" dataDxfId="56"/>
+    <tableColumn id="2" xr3:uid="{95C69B8D-1A39-40CB-B5FA-F58DC3500DA7}" name="Turno" dataDxfId="55"/>
+    <tableColumn id="3" xr3:uid="{046BEC21-BC63-4C71-8608-9399078C3481}" name="OPERADOR" dataDxfId="54"/>
+    <tableColumn id="4" xr3:uid="{C3B0A1FD-B664-4E6E-9624-C807349AADDB}" name="OBSERVAÇÃO" dataDxfId="53"/>
+    <tableColumn id="5" xr3:uid="{C7967862-84A2-4EDD-9459-5C2DFCE69540}" name="Coluna1" dataDxfId="52"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3330,7 +3333,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8AA5261E-B2CC-424C-A60F-51E466D0160F}">
-  <dimension ref="A1:S129"/>
+  <dimension ref="A1:S130"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19.7109375" style="2" customWidth="1"/>
@@ -3421,7 +3424,7 @@
       <c r="I2" s="13"/>
       <c r="J2" s="14">
         <f>AVERAGE(E2:E206)</f>
-        <v>8283.5142857142855</v>
+        <v>8268.5943396226412</v>
       </c>
       <c r="K2" s="6" t="s">
         <v>13</v>
@@ -3468,12 +3471,12 @@
       <c r="I3" s="12"/>
       <c r="K3" s="4">
         <f>SUM(E2:E2000)</f>
-        <v>869769</v>
+        <v>876471</v>
       </c>
       <c r="L3" s="4"/>
       <c r="M3" s="18">
         <f>SUM(F2:F2000)</f>
-        <v>5087</v>
+        <v>5157</v>
       </c>
       <c r="N3" s="1" t="s">
         <v>27</v>
@@ -6260,6 +6263,9 @@
       <c r="B128" s="1" t="s">
         <v>6</v>
       </c>
+      <c r="C128" s="1">
+        <v>1418443</v>
+      </c>
       <c r="D128" s="1">
         <v>8524</v>
       </c>
@@ -6287,6 +6293,32 @@
         <v>84</v>
       </c>
       <c r="H129" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="130" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A130" s="2">
+        <v>46094</v>
+      </c>
+      <c r="B130" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C130" s="1">
+        <v>1418443</v>
+      </c>
+      <c r="D130" s="1">
+        <v>8524</v>
+      </c>
+      <c r="E130" s="1">
+        <v>6702</v>
+      </c>
+      <c r="F130" s="1">
+        <v>70</v>
+      </c>
+      <c r="G130" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="H130" s="1" t="s">
         <v>17</v>
       </c>
     </row>
@@ -6397,7 +6429,7 @@
       <c r="I2" s="13"/>
       <c r="J2" s="14">
         <f>AVERAGE(E2:E206)</f>
-        <v>1519.2</v>
+        <v>1816</v>
       </c>
       <c r="K2" s="6" t="s">
         <v>13</v>
@@ -6446,12 +6478,12 @@
       <c r="J3" s="1"/>
       <c r="K3" s="4">
         <f>SUM(E2:E2000)</f>
-        <v>7596</v>
+        <v>10896</v>
       </c>
       <c r="L3" s="4"/>
       <c r="M3" s="18">
         <f>SUM(F2:F2000)</f>
-        <v>873</v>
+        <v>993</v>
       </c>
       <c r="N3" s="1" t="s">
         <v>27</v>
@@ -6615,6 +6647,24 @@
       <c r="Q7" s="1"/>
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A8" s="2">
+        <v>46094</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C8" s="1">
+        <v>1406169</v>
+      </c>
+      <c r="D8" s="1">
+        <v>8524</v>
+      </c>
+      <c r="E8" s="1">
+        <v>3300</v>
+      </c>
+      <c r="F8" s="1">
+        <v>120</v>
+      </c>
       <c r="N8" s="1" t="s">
         <v>27</v>
       </c>

</xml_diff>

<commit_message>
Atualizacao automatica (14/03/2026 16:02:43,33)
</commit_message>
<xml_diff>
--- a/Canudos.xlsx
+++ b/Canudos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PLANILHAS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{943063A0-ED43-4A30-AA3E-9F44FCBA6D38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38DB26E2-751E-4523-AC02-C658A719F2FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3585" yWindow="3585" windowWidth="21600" windowHeight="11295" xr2:uid="{2551C110-448D-4C8A-AC10-E46F4B669B16}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{2551C110-448D-4C8A-AC10-E46F4B669B16}"/>
   </bookViews>
   <sheets>
     <sheet name="ENCABEÇAMENTO" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="405" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="411" uniqueCount="96">
   <si>
     <t>OS</t>
   </si>
@@ -318,6 +318,12 @@
   </si>
   <si>
     <t xml:space="preserve">RODANDO TRANSFER E ENCABEÇADORA </t>
+  </si>
+  <si>
+    <t>MAQUINA ESTÁ APRESENTANDO PROBLEMA NA ALIMENTAÇÃO DE CANUDOS</t>
+  </si>
+  <si>
+    <t>MAQUINA DE TRANSFER APRESENTA PROBLEMA NA ALIMENTAÇÃO DE CANUDOS</t>
   </si>
 </sst>
 </file>
@@ -698,14 +704,21 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border outline="0">
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+      </border>
     </dxf>
     <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border outline="0">
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
     </dxf>
     <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -1002,6 +1015,31 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -1046,38 +1084,6 @@
         </right>
         <top/>
         <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
       </border>
     </dxf>
   </dxfs>
@@ -2953,17 +2959,17 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{5BB2D3F9-C887-4B4C-B99D-D2DF65DEC2A6}" name="Tabela5" displayName="Tabela5" ref="A1:H1048576" totalsRowCount="1" headerRowDxfId="51" dataDxfId="49" headerRowBorderDxfId="50">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{5BB2D3F9-C887-4B4C-B99D-D2DF65DEC2A6}" name="Tabela5" displayName="Tabela5" ref="A1:H1048576" totalsRowCount="1" headerRowDxfId="59" dataDxfId="57" headerRowBorderDxfId="58">
   <autoFilter ref="A1:H1048575" xr:uid="{5BB2D3F9-C887-4B4C-B99D-D2DF65DEC2A6}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{087A0113-3A7F-4ED4-85E5-B6DA7A785E6E}" name="Data" dataDxfId="48" totalsRowDxfId="7"/>
-    <tableColumn id="2" xr3:uid="{B5ACDCB9-111C-4EEF-A7F2-0DFD4B46F701}" name="Turno" dataDxfId="47" totalsRowDxfId="6"/>
-    <tableColumn id="3" xr3:uid="{8DF57E4B-CE5D-4D81-A024-AF995D46B0D6}" name="OS" dataDxfId="46" totalsRowDxfId="5"/>
-    <tableColumn id="4" xr3:uid="{ED2D14F5-1612-4387-8474-BB902D6983C6}" name="Operador" dataDxfId="45" totalsRowDxfId="4"/>
-    <tableColumn id="5" xr3:uid="{98386C95-9775-4F1F-A3CC-9A16E030AF66}" name="Produzidos" dataDxfId="44" totalsRowDxfId="3"/>
-    <tableColumn id="6" xr3:uid="{3F049097-8486-4DDD-93F7-CCC691CC4860}" name="Perdas" dataDxfId="43" totalsRowDxfId="2"/>
-    <tableColumn id="7" xr3:uid="{26B92E51-FF95-433C-9069-C56C7828476A}" name="Observação" dataDxfId="42" totalsRowDxfId="1"/>
-    <tableColumn id="8" xr3:uid="{8B43B335-323F-4C61-82F4-07648230810B}" name="Coluna1" dataDxfId="41" totalsRowDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{087A0113-3A7F-4ED4-85E5-B6DA7A785E6E}" name="Data" dataDxfId="56" totalsRowDxfId="55"/>
+    <tableColumn id="2" xr3:uid="{B5ACDCB9-111C-4EEF-A7F2-0DFD4B46F701}" name="Turno" dataDxfId="54" totalsRowDxfId="53"/>
+    <tableColumn id="3" xr3:uid="{8DF57E4B-CE5D-4D81-A024-AF995D46B0D6}" name="OS" dataDxfId="52" totalsRowDxfId="51"/>
+    <tableColumn id="4" xr3:uid="{ED2D14F5-1612-4387-8474-BB902D6983C6}" name="Operador" dataDxfId="50" totalsRowDxfId="49"/>
+    <tableColumn id="5" xr3:uid="{98386C95-9775-4F1F-A3CC-9A16E030AF66}" name="Produzidos" dataDxfId="48" totalsRowDxfId="47"/>
+    <tableColumn id="6" xr3:uid="{3F049097-8486-4DDD-93F7-CCC691CC4860}" name="Perdas" dataDxfId="46" totalsRowDxfId="45"/>
+    <tableColumn id="7" xr3:uid="{26B92E51-FF95-433C-9069-C56C7828476A}" name="Observação" dataDxfId="44" totalsRowDxfId="43"/>
+    <tableColumn id="8" xr3:uid="{8B43B335-323F-4C61-82F4-07648230810B}" name="Coluna1" dataDxfId="42" totalsRowDxfId="41"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3023,14 +3029,14 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{B6F26BC4-2F5B-4DD0-B255-2DBF5E945A60}" name="Tabela7" displayName="Tabela7" ref="A1:E1048576" totalsRowShown="0" dataDxfId="58" headerRowBorderDxfId="59" tableBorderDxfId="57">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{B6F26BC4-2F5B-4DD0-B255-2DBF5E945A60}" name="Tabela7" displayName="Tabela7" ref="A1:E1048576" totalsRowShown="0" dataDxfId="6" headerRowBorderDxfId="7" tableBorderDxfId="5">
   <autoFilter ref="A1:E1048576" xr:uid="{B6F26BC4-2F5B-4DD0-B255-2DBF5E945A60}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{A457A19A-4874-4397-B513-B6F9A3B0A60A}" name="Data" dataDxfId="56"/>
-    <tableColumn id="2" xr3:uid="{95C69B8D-1A39-40CB-B5FA-F58DC3500DA7}" name="Turno" dataDxfId="55"/>
-    <tableColumn id="3" xr3:uid="{046BEC21-BC63-4C71-8608-9399078C3481}" name="OPERADOR" dataDxfId="54"/>
-    <tableColumn id="4" xr3:uid="{C3B0A1FD-B664-4E6E-9624-C807349AADDB}" name="OBSERVAÇÃO" dataDxfId="53"/>
-    <tableColumn id="5" xr3:uid="{C7967862-84A2-4EDD-9459-5C2DFCE69540}" name="Coluna1" dataDxfId="52"/>
+    <tableColumn id="1" xr3:uid="{A457A19A-4874-4397-B513-B6F9A3B0A60A}" name="Data" dataDxfId="4"/>
+    <tableColumn id="2" xr3:uid="{95C69B8D-1A39-40CB-B5FA-F58DC3500DA7}" name="Turno" dataDxfId="3"/>
+    <tableColumn id="3" xr3:uid="{046BEC21-BC63-4C71-8608-9399078C3481}" name="OPERADOR" dataDxfId="2"/>
+    <tableColumn id="4" xr3:uid="{C3B0A1FD-B664-4E6E-9624-C807349AADDB}" name="OBSERVAÇÃO" dataDxfId="1"/>
+    <tableColumn id="5" xr3:uid="{C7967862-84A2-4EDD-9459-5C2DFCE69540}" name="Coluna1" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -6429,7 +6435,7 @@
       <c r="I2" s="13"/>
       <c r="J2" s="14">
         <f>AVERAGE(E2:E206)</f>
-        <v>1816</v>
+        <v>1711.7142857142858</v>
       </c>
       <c r="K2" s="6" t="s">
         <v>13</v>
@@ -6478,12 +6484,12 @@
       <c r="J3" s="1"/>
       <c r="K3" s="4">
         <f>SUM(E2:E2000)</f>
-        <v>10896</v>
+        <v>11982</v>
       </c>
       <c r="L3" s="4"/>
       <c r="M3" s="18">
         <f>SUM(F2:F2000)</f>
-        <v>993</v>
+        <v>1059</v>
       </c>
       <c r="N3" s="1" t="s">
         <v>27</v>
@@ -6677,6 +6683,30 @@
       <c r="Q8" s="1"/>
     </row>
     <row r="9" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A9" s="2">
+        <v>46095</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C9" s="1">
+        <v>1406169</v>
+      </c>
+      <c r="D9" s="1">
+        <v>8524</v>
+      </c>
+      <c r="E9" s="1">
+        <v>1086</v>
+      </c>
+      <c r="F9" s="1">
+        <v>66</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="H9" t="s">
+        <v>17</v>
+      </c>
       <c r="N9" s="1" t="s">
         <v>27</v>
       </c>
@@ -6925,7 +6955,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A6B5184B-1E33-47EF-9675-0892F220B5E2}">
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="4" width="23.7109375" style="1" customWidth="1"/>
@@ -6983,6 +7013,23 @@
         <v>17</v>
       </c>
     </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" s="2">
+        <v>46095</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" s="1">
+        <v>8524</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <drawing r:id="rId1"/>

</xml_diff>